<commit_message>
added in SGang Gwaay
</commit_message>
<xml_diff>
--- a/input/islands.xlsx
+++ b/input/islands.xlsx
@@ -1,6 +1,6 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="x15 xr xr6 xr10">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10212"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/robynirvine/Analyses/llgaay-gwii-20/input/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:40009_{EBEDB0EB-4C0C-914D-8313-9267A381203F}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{954348B5-F427-B444-A6A4-B31CE51E450D}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3900" yWindow="2260" windowWidth="28040" windowHeight="17440"/>
+    <workbookView xWindow="3900" yWindow="2260" windowWidth="28040" windowHeight="17440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="islands" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="21">
   <si>
     <t>Island</t>
   </si>
@@ -98,12 +98,37 @@
   <si>
     <t>T'aaxwii XaaydaGa Gwaay.yaay</t>
   </si>
+  <si>
+    <t>Sgang Gwaay Island</t>
+  </si>
+  <si>
+    <r>
+      <t>S</t>
+    </r>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri (Body)"/>
+      </rPr>
+      <t>G</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri (Body)"/>
+      </rPr>
+      <t>ang Gwaay</t>
+    </r>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="20" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="21" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -247,6 +272,12 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri (Body)"/>
+    </font>
+    <font>
+      <u/>
       <sz val="12"/>
       <color theme="1"/>
       <name val="Calibri (Body)"/>
@@ -951,8 +982,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C9"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:C10"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="27.5" bestFit="1" customWidth="1"/>
@@ -1048,6 +1079,14 @@
         <v>18</v>
       </c>
     </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>19</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>20</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>